<commit_message>
[UPDATE - 5] - Update check answer
</commit_message>
<xml_diff>
--- a/onluyen_data/69cbd7071502b2a72371f694.xlsx
+++ b/onluyen_data/69cbd7071502b2a72371f694.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Dap an" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Thong ke" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dap an" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Thong ke" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -40,6 +40,11 @@
     </font>
     <font>
       <name val="Arial"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
       <sz val="10"/>
     </font>
     <font>
@@ -47,11 +52,6 @@
       <b val="1"/>
       <color rgb="00C0392B"/>
       <sz val="12"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -86,7 +86,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -108,11 +108,44 @@
         <color rgb="00CCCCCC"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00CCCCCC"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00CCCCCC"/>
+      </left>
+      <right style="thin">
+        <color rgb="00CCCCCC"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00CCCCCC"/>
+      </left>
+      <right style="thin">
+        <color rgb="00CCCCCC"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00CCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -120,17 +153,19 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -545,6 +580,7 @@
       </c>
     </row>
     <row r="4" ht="28" customHeight="1">
+      <c r="A4" s="6" t="n"/>
       <c r="B4" s="4" t="n">
         <v>2</v>
       </c>
@@ -555,6 +591,7 @@
       </c>
     </row>
     <row r="5" ht="28" customHeight="1">
+      <c r="A5" s="6" t="n"/>
       <c r="B5" s="4" t="n">
         <v>3</v>
       </c>
@@ -565,6 +602,7 @@
       </c>
     </row>
     <row r="6" ht="28" customHeight="1">
+      <c r="A6" s="6" t="n"/>
       <c r="B6" s="4" t="n">
         <v>4</v>
       </c>
@@ -575,6 +613,7 @@
       </c>
     </row>
     <row r="7" ht="28" customHeight="1">
+      <c r="A7" s="6" t="n"/>
       <c r="B7" s="4" t="n">
         <v>5</v>
       </c>
@@ -585,6 +624,7 @@
       </c>
     </row>
     <row r="8" ht="28" customHeight="1">
+      <c r="A8" s="6" t="n"/>
       <c r="B8" s="4" t="n">
         <v>6</v>
       </c>
@@ -595,6 +635,7 @@
       </c>
     </row>
     <row r="9" ht="28" customHeight="1">
+      <c r="A9" s="6" t="n"/>
       <c r="B9" s="4" t="n">
         <v>7</v>
       </c>
@@ -605,6 +646,7 @@
       </c>
     </row>
     <row r="10" ht="28" customHeight="1">
+      <c r="A10" s="6" t="n"/>
       <c r="B10" s="4" t="n">
         <v>8</v>
       </c>
@@ -615,6 +657,7 @@
       </c>
     </row>
     <row r="11" ht="28" customHeight="1">
+      <c r="A11" s="6" t="n"/>
       <c r="B11" s="4" t="n">
         <v>9</v>
       </c>
@@ -625,6 +668,7 @@
       </c>
     </row>
     <row r="12" ht="28" customHeight="1">
+      <c r="A12" s="6" t="n"/>
       <c r="B12" s="4" t="n">
         <v>10</v>
       </c>
@@ -635,6 +679,7 @@
       </c>
     </row>
     <row r="13" ht="28" customHeight="1">
+      <c r="A13" s="6" t="n"/>
       <c r="B13" s="4" t="n">
         <v>11</v>
       </c>
@@ -645,6 +690,7 @@
       </c>
     </row>
     <row r="14" ht="28" customHeight="1">
+      <c r="A14" s="6" t="n"/>
       <c r="B14" s="4" t="n">
         <v>12</v>
       </c>
@@ -655,6 +701,7 @@
       </c>
     </row>
     <row r="15" ht="28" customHeight="1">
+      <c r="A15" s="6" t="n"/>
       <c r="B15" s="4" t="n">
         <v>13</v>
       </c>
@@ -665,6 +712,7 @@
       </c>
     </row>
     <row r="16" ht="28" customHeight="1">
+      <c r="A16" s="6" t="n"/>
       <c r="B16" s="4" t="n">
         <v>14</v>
       </c>
@@ -675,6 +723,7 @@
       </c>
     </row>
     <row r="17" ht="28" customHeight="1">
+      <c r="A17" s="6" t="n"/>
       <c r="B17" s="4" t="n">
         <v>15</v>
       </c>
@@ -685,6 +734,7 @@
       </c>
     </row>
     <row r="18" ht="28" customHeight="1">
+      <c r="A18" s="6" t="n"/>
       <c r="B18" s="4" t="n">
         <v>16</v>
       </c>
@@ -695,6 +745,7 @@
       </c>
     </row>
     <row r="19" ht="28" customHeight="1">
+      <c r="A19" s="6" t="n"/>
       <c r="B19" s="4" t="n">
         <v>17</v>
       </c>
@@ -705,6 +756,7 @@
       </c>
     </row>
     <row r="20" ht="28" customHeight="1">
+      <c r="A20" s="6" t="n"/>
       <c r="B20" s="4" t="n">
         <v>18</v>
       </c>
@@ -715,6 +767,7 @@
       </c>
     </row>
     <row r="21" ht="28" customHeight="1">
+      <c r="A21" s="6" t="n"/>
       <c r="B21" s="4" t="n">
         <v>19</v>
       </c>
@@ -725,6 +778,7 @@
       </c>
     </row>
     <row r="22" ht="28" customHeight="1">
+      <c r="A22" s="6" t="n"/>
       <c r="B22" s="4" t="n">
         <v>20</v>
       </c>
@@ -735,6 +789,7 @@
       </c>
     </row>
     <row r="23" ht="28" customHeight="1">
+      <c r="A23" s="6" t="n"/>
       <c r="B23" s="4" t="n">
         <v>21</v>
       </c>
@@ -745,6 +800,7 @@
       </c>
     </row>
     <row r="24" ht="28" customHeight="1">
+      <c r="A24" s="6" t="n"/>
       <c r="B24" s="4" t="n">
         <v>22</v>
       </c>
@@ -755,6 +811,7 @@
       </c>
     </row>
     <row r="25" ht="28" customHeight="1">
+      <c r="A25" s="6" t="n"/>
       <c r="B25" s="4" t="n">
         <v>23</v>
       </c>
@@ -765,6 +822,7 @@
       </c>
     </row>
     <row r="26" ht="28" customHeight="1">
+      <c r="A26" s="6" t="n"/>
       <c r="B26" s="4" t="n">
         <v>24</v>
       </c>
@@ -775,6 +833,7 @@
       </c>
     </row>
     <row r="27" ht="28" customHeight="1">
+      <c r="A27" s="6" t="n"/>
       <c r="B27" s="4" t="n">
         <v>25</v>
       </c>
@@ -785,6 +844,7 @@
       </c>
     </row>
     <row r="28" ht="28" customHeight="1">
+      <c r="A28" s="6" t="n"/>
       <c r="B28" s="4" t="n">
         <v>26</v>
       </c>
@@ -795,6 +855,7 @@
       </c>
     </row>
     <row r="29" ht="28" customHeight="1">
+      <c r="A29" s="6" t="n"/>
       <c r="B29" s="4" t="n">
         <v>27</v>
       </c>
@@ -805,6 +866,7 @@
       </c>
     </row>
     <row r="30" ht="28" customHeight="1">
+      <c r="A30" s="6" t="n"/>
       <c r="B30" s="4" t="n">
         <v>28</v>
       </c>
@@ -815,6 +877,7 @@
       </c>
     </row>
     <row r="31" ht="28" customHeight="1">
+      <c r="A31" s="6" t="n"/>
       <c r="B31" s="4" t="n">
         <v>29</v>
       </c>
@@ -825,6 +888,7 @@
       </c>
     </row>
     <row r="32" ht="28" customHeight="1">
+      <c r="A32" s="6" t="n"/>
       <c r="B32" s="4" t="n">
         <v>30</v>
       </c>
@@ -835,6 +899,7 @@
       </c>
     </row>
     <row r="33" ht="28" customHeight="1">
+      <c r="A33" s="6" t="n"/>
       <c r="B33" s="4" t="n">
         <v>31</v>
       </c>
@@ -845,6 +910,7 @@
       </c>
     </row>
     <row r="34" ht="28" customHeight="1">
+      <c r="A34" s="6" t="n"/>
       <c r="B34" s="4" t="n">
         <v>32</v>
       </c>
@@ -855,6 +921,7 @@
       </c>
     </row>
     <row r="35" ht="28" customHeight="1">
+      <c r="A35" s="6" t="n"/>
       <c r="B35" s="4" t="n">
         <v>33</v>
       </c>
@@ -865,6 +932,7 @@
       </c>
     </row>
     <row r="36" ht="28" customHeight="1">
+      <c r="A36" s="6" t="n"/>
       <c r="B36" s="4" t="n">
         <v>34</v>
       </c>
@@ -875,6 +943,7 @@
       </c>
     </row>
     <row r="37" ht="28" customHeight="1">
+      <c r="A37" s="6" t="n"/>
       <c r="B37" s="4" t="n">
         <v>35</v>
       </c>
@@ -885,6 +954,7 @@
       </c>
     </row>
     <row r="38" ht="28" customHeight="1">
+      <c r="A38" s="6" t="n"/>
       <c r="B38" s="4" t="n">
         <v>36</v>
       </c>
@@ -895,6 +965,7 @@
       </c>
     </row>
     <row r="39" ht="28" customHeight="1">
+      <c r="A39" s="6" t="n"/>
       <c r="B39" s="4" t="n">
         <v>37</v>
       </c>
@@ -905,6 +976,7 @@
       </c>
     </row>
     <row r="40" ht="28" customHeight="1">
+      <c r="A40" s="6" t="n"/>
       <c r="B40" s="4" t="n">
         <v>38</v>
       </c>
@@ -915,6 +987,7 @@
       </c>
     </row>
     <row r="41" ht="28" customHeight="1">
+      <c r="A41" s="6" t="n"/>
       <c r="B41" s="4" t="n">
         <v>39</v>
       </c>
@@ -925,6 +998,7 @@
       </c>
     </row>
     <row r="42" ht="28" customHeight="1">
+      <c r="A42" s="7" t="n"/>
       <c r="B42" s="4" t="n">
         <v>40</v>
       </c>
@@ -958,37 +1032,37 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="6" t="inlineStr">
+      <c r="A1" s="8" t="inlineStr">
         <is>
           <t>Dang cau</t>
         </is>
       </c>
-      <c r="B1" s="6" t="inlineStr">
+      <c r="B1" s="8" t="inlineStr">
         <is>
           <t>So luong</t>
         </is>
       </c>
-      <c r="C1" s="6" t="inlineStr">
+      <c r="C1" s="8" t="inlineStr">
         <is>
           <t>Tong diem</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="7" t="inlineStr">
+      <c r="A2" s="9" t="inlineStr">
         <is>
           <t>Trac nghiem</t>
         </is>
       </c>
-      <c r="B2" s="7" t="n">
+      <c r="B2" s="9" t="n">
         <v>40</v>
       </c>
-      <c r="C2" s="7" t="n">
+      <c r="C2" s="9" t="n">
         <v>10</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="inlineStr">
+      <c r="A3" s="10" t="inlineStr">
         <is>
           <t>TONG</t>
         </is>

</xml_diff>